<commit_message>
committed @ 2025-10-21-233045-0500 by tychen@TYCMBA.local
</commit_message>
<xml_diff>
--- a/data/Excel_Sample.xlsx
+++ b/data/Excel_Sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,36 +425,46 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G5"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.3</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.2</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -474,12 +484,18 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
+        <v>0</v>
+      </c>
+      <c r="F2" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" t="n">
         <v>1</v>
       </c>
-      <c r="F2" t="n">
+      <c r="H2" t="n">
         <v>2</v>
       </c>
-      <c r="G2" t="n">
+      <c r="I2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -494,15 +510,21 @@
         <v>1</v>
       </c>
       <c r="D3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="n">
         <v>4</v>
       </c>
-      <c r="E3" t="n">
+      <c r="G3" t="n">
         <v>5</v>
       </c>
-      <c r="F3" t="n">
+      <c r="H3" t="n">
         <v>6</v>
       </c>
-      <c r="G3" t="n">
+      <c r="I3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -517,15 +539,21 @@
         <v>2</v>
       </c>
       <c r="D4" t="n">
+        <v>2</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2</v>
+      </c>
+      <c r="F4" t="n">
         <v>8</v>
       </c>
-      <c r="E4" t="n">
+      <c r="G4" t="n">
         <v>9</v>
       </c>
-      <c r="F4" t="n">
+      <c r="H4" t="n">
         <v>10</v>
       </c>
-      <c r="G4" t="n">
+      <c r="I4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -540,15 +568,21 @@
         <v>3</v>
       </c>
       <c r="D5" t="n">
+        <v>3</v>
+      </c>
+      <c r="E5" t="n">
+        <v>3</v>
+      </c>
+      <c r="F5" t="n">
         <v>12</v>
       </c>
-      <c r="E5" t="n">
+      <c r="G5" t="n">
         <v>13</v>
       </c>
-      <c r="F5" t="n">
+      <c r="H5" t="n">
         <v>14</v>
       </c>
-      <c r="G5" t="n">
+      <c r="I5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
committed @ 2026-01-23-002455-0600 by tychen@TYCMBA.local
</commit_message>
<xml_diff>
--- a/data/Excel_Sample.xlsx
+++ b/data/Excel_Sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,46 +425,51 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:J5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.4</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -490,12 +495,15 @@
         <v>0</v>
       </c>
       <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
         <v>1</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>2</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -516,15 +524,18 @@
         <v>1</v>
       </c>
       <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
         <v>4</v>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>5</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>6</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -545,15 +556,18 @@
         <v>2</v>
       </c>
       <c r="F4" t="n">
+        <v>2</v>
+      </c>
+      <c r="G4" t="n">
         <v>8</v>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>9</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>10</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -574,15 +588,18 @@
         <v>3</v>
       </c>
       <c r="F5" t="n">
+        <v>3</v>
+      </c>
+      <c r="G5" t="n">
         <v>12</v>
       </c>
-      <c r="G5" t="n">
+      <c r="H5" t="n">
         <v>13</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>14</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
committed @ 2026-02-16-023021-0600 by tychen@TYCMBA.local
</commit_message>
<xml_diff>
--- a/data/Excel_Sample.xlsx
+++ b/data/Excel_Sample.xlsx
@@ -425,51 +425,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.5</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0.4</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -498,12 +503,15 @@
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -527,15 +535,18 @@
         <v>1</v>
       </c>
       <c r="G3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H3" t="n">
         <v>4</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>5</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>6</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -559,15 +570,18 @@
         <v>2</v>
       </c>
       <c r="G4" t="n">
+        <v>2</v>
+      </c>
+      <c r="H4" t="n">
         <v>8</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>9</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>10</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -591,15 +605,18 @@
         <v>3</v>
       </c>
       <c r="G5" t="n">
+        <v>3</v>
+      </c>
+      <c r="H5" t="n">
         <v>12</v>
       </c>
-      <c r="H5" t="n">
+      <c r="I5" t="n">
         <v>13</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>14</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
committed @ 2026-02-16-024645-0600 by tychen@TYCMBA.local
</commit_message>
<xml_diff>
--- a/data/Excel_Sample.xlsx
+++ b/data/Excel_Sample.xlsx
@@ -425,56 +425,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K5"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.6</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0.5</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.4</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -506,12 +511,15 @@
         <v>0</v>
       </c>
       <c r="I2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2" t="n">
+        <v>2</v>
+      </c>
+      <c r="L2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -538,15 +546,18 @@
         <v>1</v>
       </c>
       <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
         <v>4</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>5</v>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>6</v>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -573,15 +584,18 @@
         <v>2</v>
       </c>
       <c r="H4" t="n">
+        <v>2</v>
+      </c>
+      <c r="I4" t="n">
         <v>8</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>9</v>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>10</v>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -608,15 +622,18 @@
         <v>3</v>
       </c>
       <c r="H5" t="n">
+        <v>3</v>
+      </c>
+      <c r="I5" t="n">
         <v>12</v>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>13</v>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>14</v>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
committed @ 2026-02-16-030658-0600 by tychen@TYCMBA.local
</commit_message>
<xml_diff>
--- a/data/Excel_Sample.xlsx
+++ b/data/Excel_Sample.xlsx
@@ -425,61 +425,71 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L5"/>
+  <dimension ref="A1:N5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.8</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Unnamed: 0.7</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0.6</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.5</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.4</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -514,12 +524,18 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K2" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -549,15 +565,21 @@
         <v>1</v>
       </c>
       <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" t="n">
         <v>4</v>
       </c>
-      <c r="J3" t="n">
+      <c r="L3" t="n">
         <v>5</v>
       </c>
-      <c r="K3" t="n">
+      <c r="M3" t="n">
         <v>6</v>
       </c>
-      <c r="L3" t="n">
+      <c r="N3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -587,15 +609,21 @@
         <v>2</v>
       </c>
       <c r="I4" t="n">
+        <v>2</v>
+      </c>
+      <c r="J4" t="n">
+        <v>2</v>
+      </c>
+      <c r="K4" t="n">
         <v>8</v>
       </c>
-      <c r="J4" t="n">
+      <c r="L4" t="n">
         <v>9</v>
       </c>
-      <c r="K4" t="n">
+      <c r="M4" t="n">
         <v>10</v>
       </c>
-      <c r="L4" t="n">
+      <c r="N4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -625,15 +653,21 @@
         <v>3</v>
       </c>
       <c r="I5" t="n">
+        <v>3</v>
+      </c>
+      <c r="J5" t="n">
+        <v>3</v>
+      </c>
+      <c r="K5" t="n">
         <v>12</v>
       </c>
-      <c r="J5" t="n">
+      <c r="L5" t="n">
         <v>13</v>
       </c>
-      <c r="K5" t="n">
+      <c r="M5" t="n">
         <v>14</v>
       </c>
-      <c r="L5" t="n">
+      <c r="N5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
committed @ 2026-02-16-092725+0000 by tychen@ubuntu
</commit_message>
<xml_diff>
--- a/data/Excel_Sample.xlsx
+++ b/data/Excel_Sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,71 +425,76 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N5"/>
+  <dimension ref="A1:O5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.9</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0.8</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.7</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.6</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.5</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.4</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -530,12 +535,15 @@
         <v>0</v>
       </c>
       <c r="L2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="N2" t="n">
+        <v>2</v>
+      </c>
+      <c r="O2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -571,15 +579,18 @@
         <v>1</v>
       </c>
       <c r="K3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L3" t="n">
         <v>4</v>
       </c>
-      <c r="L3" t="n">
+      <c r="M3" t="n">
         <v>5</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>6</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -615,15 +626,18 @@
         <v>2</v>
       </c>
       <c r="K4" t="n">
+        <v>2</v>
+      </c>
+      <c r="L4" t="n">
         <v>8</v>
       </c>
-      <c r="L4" t="n">
+      <c r="M4" t="n">
         <v>9</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>10</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -659,15 +673,18 @@
         <v>3</v>
       </c>
       <c r="K5" t="n">
+        <v>3</v>
+      </c>
+      <c r="L5" t="n">
         <v>12</v>
       </c>
-      <c r="L5" t="n">
+      <c r="M5" t="n">
         <v>13</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>14</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
committed @ 2026-02-16-094826+0000 by tychen@ubuntu
</commit_message>
<xml_diff>
--- a/data/Excel_Sample.xlsx
+++ b/data/Excel_Sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,76 +425,81 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O5"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.10</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0.9</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.8</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.7</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.6</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.5</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.4</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -538,12 +543,15 @@
         <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2" t="n">
+        <v>2</v>
+      </c>
+      <c r="P2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -582,15 +590,18 @@
         <v>1</v>
       </c>
       <c r="L3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M3" t="n">
         <v>4</v>
       </c>
-      <c r="M3" t="n">
+      <c r="N3" t="n">
         <v>5</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>6</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -629,15 +640,18 @@
         <v>2</v>
       </c>
       <c r="L4" t="n">
+        <v>2</v>
+      </c>
+      <c r="M4" t="n">
         <v>8</v>
       </c>
-      <c r="M4" t="n">
+      <c r="N4" t="n">
         <v>9</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>10</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -676,15 +690,18 @@
         <v>3</v>
       </c>
       <c r="L5" t="n">
+        <v>3</v>
+      </c>
+      <c r="M5" t="n">
         <v>12</v>
       </c>
-      <c r="M5" t="n">
+      <c r="N5" t="n">
         <v>13</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>14</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
committed @ 2026-02-16-160530-0600 by tcn85@rtsjpl774kw20.managed.mst.edu
</commit_message>
<xml_diff>
--- a/data/Excel_Sample.xlsx
+++ b/data/Excel_Sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,81 +425,86 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P5"/>
+  <dimension ref="A1:Q5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.11</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0.10</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.9</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.8</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.7</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.6</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.5</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.4</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -546,12 +551,15 @@
         <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="P2" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -593,15 +601,18 @@
         <v>1</v>
       </c>
       <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
         <v>4</v>
       </c>
-      <c r="N3" t="n">
+      <c r="O3" t="n">
         <v>5</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>6</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -643,15 +654,18 @@
         <v>2</v>
       </c>
       <c r="M4" t="n">
+        <v>2</v>
+      </c>
+      <c r="N4" t="n">
         <v>8</v>
       </c>
-      <c r="N4" t="n">
+      <c r="O4" t="n">
         <v>9</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>10</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -693,15 +707,18 @@
         <v>3</v>
       </c>
       <c r="M5" t="n">
+        <v>3</v>
+      </c>
+      <c r="N5" t="n">
         <v>12</v>
       </c>
-      <c r="N5" t="n">
+      <c r="O5" t="n">
         <v>13</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>14</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
committed @ 2026-02-16-220724+0000 by tychen@ubuntu
</commit_message>
<xml_diff>
--- a/data/Excel_Sample.xlsx
+++ b/data/Excel_Sample.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,86 +425,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q5"/>
+  <dimension ref="A1:R5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.12</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0.11</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.10</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.9</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.8</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.7</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.6</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.5</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.4</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -554,12 +559,15 @@
         <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q2" t="n">
+        <v>2</v>
+      </c>
+      <c r="R2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -604,15 +612,18 @@
         <v>1</v>
       </c>
       <c r="N3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" t="n">
         <v>4</v>
       </c>
-      <c r="O3" t="n">
+      <c r="P3" t="n">
         <v>5</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>6</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -657,15 +668,18 @@
         <v>2</v>
       </c>
       <c r="N4" t="n">
+        <v>2</v>
+      </c>
+      <c r="O4" t="n">
         <v>8</v>
       </c>
-      <c r="O4" t="n">
+      <c r="P4" t="n">
         <v>9</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>10</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -710,15 +724,18 @@
         <v>3</v>
       </c>
       <c r="N5" t="n">
+        <v>3</v>
+      </c>
+      <c r="O5" t="n">
         <v>12</v>
       </c>
-      <c r="O5" t="n">
+      <c r="P5" t="n">
         <v>13</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>14</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>

<commit_message>
committed @ 2026-02-18-162759-0600 by tcn85@rtsjpl774kw20.managed.mst.edu
</commit_message>
<xml_diff>
--- a/data/Excel_Sample.xlsx
+++ b/data/Excel_Sample.xlsx
@@ -425,91 +425,96 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R5"/>
+  <dimension ref="A1:S5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>Unnamed: 0.13</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Unnamed: 0.12</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.11</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.10</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.9</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.8</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.7</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.6</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.5</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.4</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.3</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.2</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0.1</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Unnamed: 0</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>a</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>b</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>c</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>d</t>
         </is>
@@ -562,12 +567,15 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R2" t="n">
+        <v>2</v>
+      </c>
+      <c r="S2" t="n">
         <v>3</v>
       </c>
     </row>
@@ -615,15 +623,18 @@
         <v>1</v>
       </c>
       <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
         <v>4</v>
       </c>
-      <c r="P3" t="n">
+      <c r="Q3" t="n">
         <v>5</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="R3" t="n">
         <v>6</v>
       </c>
-      <c r="R3" t="n">
+      <c r="S3" t="n">
         <v>7</v>
       </c>
     </row>
@@ -671,15 +682,18 @@
         <v>2</v>
       </c>
       <c r="O4" t="n">
+        <v>2</v>
+      </c>
+      <c r="P4" t="n">
         <v>8</v>
       </c>
-      <c r="P4" t="n">
+      <c r="Q4" t="n">
         <v>9</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="R4" t="n">
         <v>10</v>
       </c>
-      <c r="R4" t="n">
+      <c r="S4" t="n">
         <v>11</v>
       </c>
     </row>
@@ -727,15 +741,18 @@
         <v>3</v>
       </c>
       <c r="O5" t="n">
+        <v>3</v>
+      </c>
+      <c r="P5" t="n">
         <v>12</v>
       </c>
-      <c r="P5" t="n">
+      <c r="Q5" t="n">
         <v>13</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="R5" t="n">
         <v>14</v>
       </c>
-      <c r="R5" t="n">
+      <c r="S5" t="n">
         <v>15</v>
       </c>
     </row>

</xml_diff>